<commit_message>
Reset LFHVM to 1
</commit_message>
<xml_diff>
--- a/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
+++ b/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\elec\LFHVM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\LFHVM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB475A61-37DD-4079-87FF-63CDE72F6CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15058F08-C0EF-407C-A6A9-8D93573F6431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23640" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -227,9 +227,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -267,7 +267,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -373,7 +373,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -515,7 +515,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -524,17 +524,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AFABDF-6A59-4ED9-8641-463A0343EC57}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="43.140625" customWidth="1"/>
+    <col min="2" max="2" width="43.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -542,67 +542,67 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
         <v>2021</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -622,13 +622,13 @@
     <tabColor theme="8" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="9" width="16.28515625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" customWidth="1"/>
+    <col min="2" max="9" width="16.26953125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>27</v>
       </c>
@@ -657,178 +657,178 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="C2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="D2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="E2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="F2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="G2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H2" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="I2" s="6">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="C3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="D3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="E3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="F3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="G3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H3" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="I3" s="6">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="C4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="D4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="E4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="F4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="G4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H4" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="I4" s="6">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="C5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="D5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="E5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="F5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H5" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="I5" s="6">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
       <c r="B6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="C6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="D6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="E6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="F6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="G6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H6" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="I6" s="6">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="C7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="D7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="E7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="G7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="I7" s="6">
-        <v>0.64</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated SHELF/SYSHECF files from Robbie
</commit_message>
<xml_diff>
--- a/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
+++ b/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\LFHVM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\LFHVM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9909905-9A1D-4E32-BB0B-0DE2A91A16D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BCD82B-854C-4C9D-B0F7-D4DF5E217A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
+    <workbookView xWindow="-25425" yWindow="2115" windowWidth="23160" windowHeight="13560" activeTab="1" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -530,17 +530,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AFABDF-6A59-4ED9-8641-463A0343EC57}">
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="43.1796875" customWidth="1"/>
+    <col min="2" max="2" width="43.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -548,77 +548,77 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
         <v>2021</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -638,13 +638,13 @@
     <tabColor theme="8" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.453125" customWidth="1"/>
-    <col min="2" max="9" width="16.26953125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="9" width="16.28515625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>27</v>
       </c>
@@ -673,7 +673,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -684,10 +684,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E2" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F2" s="6">
         <v>1</v>
@@ -702,7 +702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -713,10 +713,10 @@
         <v>1</v>
       </c>
       <c r="D3" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E3" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F3" s="6">
         <v>1</v>
@@ -731,7 +731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -742,10 +742,10 @@
         <v>1</v>
       </c>
       <c r="D4" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E4" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F4" s="6">
         <v>1</v>
@@ -760,7 +760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -771,10 +771,10 @@
         <v>1</v>
       </c>
       <c r="D5" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E5" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F5" s="6">
         <v>1</v>
@@ -789,7 +789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -800,10 +800,10 @@
         <v>1</v>
       </c>
       <c r="D6" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E6" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F6" s="6">
         <v>1</v>
@@ -818,7 +818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -829,10 +829,10 @@
         <v>1</v>
       </c>
       <c r="D7" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E7" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6">
         <v>1</v>

</xml_diff>